<commit_message>
Accept NaughtyStrings snapshots for OpenXmlHtml 1.7.4
OpenXmlHtml 1.7.4 no longer treats whitespace at the edge of a block as content, so the html column of two rows lost its edge spaces.
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/NaughtyStringsTests.Test.verified.xlsx
+++ b/src/Excelsior.Tests/NaughtyStringsTests.Test.verified.xlsx
@@ -6581,7 +6581,7 @@
             <rPr>
               <u/>
             </rPr>
-            <t xml:space="preserve"> Copy me</t>
+            <t xml:space="preserve">Copy me</t>
           </r>
         </is>
       </c>
@@ -6598,7 +6598,7 @@
             <rPr>
               <i/>
             </rPr>
-            <t xml:space="preserve"> Scroll over me </t>
+            <t xml:space="preserve">Scroll over me</t>
           </r>
         </is>
       </c>

</xml_diff>